<commit_message>
chore: Modify Icon mapping svg file naming
</commit_message>
<xml_diff>
--- a/data/import_label_data.xlsx
+++ b/data/import_label_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/Junyuan_Workspace/coding_space/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D73B42D-904B-8840-A8FE-F23F811FC87D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7283700B-9932-6946-99D8-99F6A95C913E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -379,12 +379,6 @@
     <t>Washing Guide</t>
   </si>
   <si>
-    <t>DO NOT BLEACH
-DO NOT TUMBLE DRY
-DO NOT IRON
-DO NOT DRY CLEAN</t>
-  </si>
-  <si>
     <t>Seat Cushion Cover
 Primary Fabric:
 100%POLYESTER
@@ -447,13 +441,21 @@
     </r>
   </si>
   <si>
-    <t>WASH WITH COLD WATER GENTLY
+    <t>Y</t>
+  </si>
+  <si>
+    <t>DO NOT BLEACH
+DO NOT TUMBLE DRY
+DO NOT IRON
+HAND WASH SEPARATELY BELOW 30°C 
+HAND -WASH ONLY</t>
+  </si>
+  <si>
+    <t>WASH WITH COLD WATER
 DO NOT DRY CLEAN 
 DO NOT BLEACH
-IRON WITH LOW HEAT</t>
-  </si>
-  <si>
-    <t>Y</t>
+IRONING WITH LOW HEAT
+IRON ANY TEMP, STEAM</t>
   </si>
 </sst>
 </file>
@@ -992,7 +994,7 @@
         <v>35</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="230.5" customHeight="1">
@@ -1000,7 +1002,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>15</v>
@@ -1015,13 +1017,13 @@
         <v>28</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="I2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="169.5" customHeight="1">
@@ -1044,10 +1046,10 @@
         <v>31</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="169.5" customHeight="1">

</xml_diff>

<commit_message>
feat: Adjust SVG text alignment and enable text-only display for specific washing instructions.
</commit_message>
<xml_diff>
--- a/data/import_label_data.xlsx
+++ b/data/import_label_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/Junyuan_Workspace/coding_space/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7283700B-9932-6946-99D8-99F6A95C913E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E34DCA2-1707-BB48-9F96-543007EE7690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -453,7 +453,7 @@
   <si>
     <t>WASH WITH COLD WATER
 DO NOT DRY CLEAN 
-DO NOT BLEACH
+SPOT CLEAN
 IRONING WITH LOW HEAT
 IRON ANY TEMP, STEAM</t>
   </si>

</xml_diff>

<commit_message>
feat: implement dynamic SVG resizing for Label 2 based on material text length and update validation logic to support label-specific requirements.
</commit_message>
<xml_diff>
--- a/data/import_label_data.xlsx
+++ b/data/import_label_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/Junyuan_Workspace/coding_space/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E34DCA2-1707-BB48-9F96-543007EE7690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F411BC-A5F2-8942-8B7C-5B9ABA795A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,60 +77,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">BODY (ARMREST) :
-95% POLYURETHANE FOAM PAD
-5% POLYESTER FIBER BATTING
-PILLOW BOLSTERS (2):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>100% POLYESTER FIBER</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EC1103 ottoman</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">
-BODY (OTTOMAN)
-95% POLYURETHANE FOAM PAD
-5% POLYESTER FIBER BATTING
-SEAT CUSHION(1)
-80% POLYURETHANE FOAM PAD
-15% </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>POLYESTER FIBER</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-5% POLYESTER FIBER BATTING</t>
-    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -455,7 +402,59 @@
 DO NOT DRY CLEAN 
 SPOT CLEAN
 IRONING WITH LOW HEAT
-IRON ANY TEMP, STEAM</t>
+IRON ANY TEMP, STEAM
+Note: Washing reduces spill-resistant finish over time. Spot clean recommended</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+BODY (OTTOMAN)
+95% POLYURETHANE FOAM PAD
+5% POLYESTER FIBER BATTING
+SEAT CUSHION(1)
+80% POLYURETHANE FOAM PAD POLYURETHANE FOAM PAD
+15% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>POLYESTER FIBER</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+5% POLYESTER FIBER BATTING</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BODY (ARMREST) :
+95% POLYURETHANE FOAM PAD
+5% POLYESTER FIBER BATTINGPOLYESTER FIBER BATTINGPOLYESTER FIBER BATTINGATTINGPOLYESTER FIBER BATTINGPOLYESTER FIBER BATTINGATTINGPOLYESTER FIBER BATTINGPOLYESTER FIBER BATTING
+PILLOW BOLSTERS (2):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>100% POLYESTER FIBER</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -979,22 +978,22 @@
         <v>2</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="10" t="s">
-        <v>18</v>
-      </c>
       <c r="F1" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H1" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="11" t="s">
         <v>35</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="230.5" customHeight="1">
@@ -1002,28 +1001,28 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>40</v>
-      </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="169.5" customHeight="1">
@@ -1031,130 +1030,130 @@
         <v>4</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="169.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="169.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="169.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="169.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="169.5" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="169.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: centralize origin country mapping in term_config and update label generation scripts to use the shared dictionary
</commit_message>
<xml_diff>
--- a/data/import_label_data.xlsx
+++ b/data/import_label_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/Junyuan_Workspace/coding_space/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F411BC-A5F2-8942-8B7C-5B9ABA795A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC0BEA3-CA48-4E4F-A4D0-64E878D26E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
   <si>
     <t>default_code</t>
   </si>
@@ -265,10 +265,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Origin (CN/VN/KHM)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>KHM</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -455,6 +451,12 @@
       </rPr>
       <t>100% POLYESTER FIBER</t>
     </r>
+  </si>
+  <si>
+    <t>Origin (CN/VN/KHM/US)</t>
+  </si>
+  <si>
+    <t>US</t>
   </si>
 </sst>
 </file>
@@ -984,16 +986,16 @@
         <v>16</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="G1" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="11" t="s">
-        <v>33</v>
-      </c>
       <c r="I1" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="230.5" customHeight="1">
@@ -1001,7 +1003,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>13</v>
@@ -1013,16 +1015,16 @@
         <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="169.5" customHeight="1">
@@ -1030,7 +1032,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>13</v>
@@ -1042,13 +1044,13 @@
         <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="169.5" customHeight="1">
@@ -1056,7 +1058,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>19</v>
@@ -1082,7 +1084,7 @@
         <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="169.5" customHeight="1">
@@ -1127,7 +1129,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>23</v>
@@ -1144,7 +1146,7 @@
         <v>12</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>24</v>
@@ -1159,8 +1161,8 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" imeMode="off" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F1048576" xr:uid="{A7A594BB-3937-FA4A-84CC-7EE2D273797F}">
-      <formula1>"CN, VN, KHM"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{A7A594BB-3937-FA4A-84CC-7EE2D273797F}">
+      <formula1>"CN, VN, KHM, US"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E1048576" xr:uid="{F312475C-390A-5143-85D6-61D8E4B0F0B1}">
       <formula1>"Mopio,Castlery"</formula1>

</xml_diff>

<commit_message>
feat: make registration number optional for Label 2 and update validation logic accordingly
</commit_message>
<xml_diff>
--- a/data/import_label_data.xlsx
+++ b/data/import_label_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/planet.cat/Documents/Junyuan_Workspace/coding_space/label_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC0BEA3-CA48-4E4F-A4D0-64E878D26E74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84576CF-E69A-984E-9726-7DE6B6A56525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="42">
   <si>
     <t>default_code</t>
   </si>
@@ -195,9 +195,6 @@
   <si>
     <t>Castlery</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RI-17530 (VN)</t>
   </si>
   <si>
     <t>RI-17531 (VN)</t>
@@ -986,16 +983,16 @@
         <v>16</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G1" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="11" t="s">
-        <v>32</v>
-      </c>
       <c r="I1" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="230.5" customHeight="1">
@@ -1003,7 +1000,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>13</v>
@@ -1015,16 +1012,16 @@
         <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="169.5" customHeight="1">
@@ -1032,11 +1029,9 @@
         <v>4</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C3" s="5"/>
       <c r="D3" t="s">
         <v>15</v>
       </c>
@@ -1044,13 +1039,13 @@
         <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="169.5" customHeight="1">
@@ -1058,16 +1053,20 @@
         <v>5</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>19</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="C4" s="5"/>
       <c r="E4" t="s">
         <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="169.5" customHeight="1">
@@ -1078,13 +1077,19 @@
         <v>7</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5" t="s">
         <v>18</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="169.5" customHeight="1">
@@ -1095,13 +1100,19 @@
         <v>9</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
         <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="169.5" customHeight="1">
@@ -1109,10 +1120,10 @@
         <v>10</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>15</v>
@@ -1121,7 +1132,13 @@
         <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>26</v>
+        <v>25</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="169.5" customHeight="1">
@@ -1129,16 +1146,22 @@
         <v>11</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>25</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="169.5" customHeight="1">
@@ -1146,16 +1169,22 @@
         <v>12</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" t="s">
         <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>